<commit_message>
paper run 2026-08-31 11:47
</commit_message>
<xml_diff>
--- a/reports/2026-08-31.xlsx
+++ b/reports/2026-08-31.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,1210 @@
       </c>
       <c r="K3" t="n">
         <v>4.89</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:09:28.393980+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00131</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:11:17.134358+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:24:26.004067+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="G6" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00121</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>5.63</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:26:15.932760+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00344</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>5.63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:28:48.848286+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="G8" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.00101</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>5.89</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:44:11.026886+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="G9" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.00103</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:44:28.732028+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.00131</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:57:22.703590+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="G11" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.00117</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>7.06</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-31T07:59:25.325721+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.797</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>7.06</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:09:26.602960+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="G13" t="n">
+        <v>15.81</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.797</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.00102</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>7.75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:11:45.190244+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="G14" t="n">
+        <v>15.81</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.00107</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>-8.06</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:26:16.951944+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="G15" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0.00113</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:28:46.769176+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.00205</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:33:54.986242+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="G17" t="n">
+        <v>17.29</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>8.470000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:41:15.541297+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F18" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="G18" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.00113</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>8.880000000000001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:43:46.644119+00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F19" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="G19" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.00269</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>8.880000000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:49:11.093610+00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="G20" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.00102</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>9.73</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:53:45.966392+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="G21" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.00101</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:56:15.946032+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F22" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="G22" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.00128</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-31T08:58:45.610222+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F23" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="G23" t="n">
+        <v>21.82</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>10.69</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:08:46.185349+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="G24" t="n">
+        <v>23.87</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.00243</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:11:16.183342+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>15</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F25" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="G25" t="n">
+        <v>23.87</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.00196</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:18:45.660473+00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F26" t="n">
+        <v>13.34</v>
+      </c>
+      <c r="G26" t="n">
+        <v>26.16</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>12.82</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:23:46.935745+00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F27" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="G27" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.00126</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>13.44</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:26:17.157252+00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>15</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F28" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.00142</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>13.44</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:13:45.906309+00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F29" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="G29" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.769</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.00145</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>14.72</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:13:47.506005+00:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F30" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="G30" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.00113</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>14.72</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:28:45.511115+00:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F31" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="G31" t="n">
+        <v>32.94</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>16.14</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +1775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +1797,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +1807,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -613,7 +1817,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -623,7 +1827,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.9666666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +1837,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.390000000000001</v>
+        <v>254.7</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +1847,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9.390000000000001</v>
+        <v>262.76</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +1857,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-8.06</v>
       </c>
     </row>
     <row r="9">
@@ -663,7 +1867,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +1877,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>106.81</v>
+        <v>352.1199999999999</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +1928,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="D15" t="n">
-        <v>22.33</v>
+        <v>186.6</v>
       </c>
       <c r="E15" t="n">
-        <v>9.390000000000001</v>
+        <v>92.27</v>
       </c>
     </row>
     <row r="16">
@@ -743,16 +1947,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="D16" t="n">
-        <v>18.35</v>
+        <v>349.58</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>162.43</v>
       </c>
     </row>
     <row r="17">
@@ -769,16 +1973,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D18" t="n">
-        <v>4.5</v>
+        <v>142.49</v>
       </c>
       <c r="E18" t="n">
-        <v>4.5</v>
+        <v>67.66</v>
       </c>
     </row>
     <row r="19">
@@ -788,86 +1992,86 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D19" t="n">
-        <v>9.74</v>
+        <v>143.76</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>60.11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>26.44</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>4.89</v>
+        <v>55.62</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>22</v>
+      </c>
+      <c r="C21" t="n">
+        <v>21</v>
+      </c>
+      <c r="D21" t="n">
+        <v>157.89</v>
+      </c>
+      <c r="E21" t="n">
+        <v>71.31</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>7</v>
-      </c>
-      <c r="C22" t="n">
-        <v>7</v>
-      </c>
-      <c r="D22" t="n">
-        <v>34.05</v>
-      </c>
-      <c r="E22" t="n">
-        <v>9.390000000000001</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D23" t="n">
-        <v>3.43</v>
+        <v>529.55</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>254.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -877,7 +2081,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -886,329 +2090,527 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>7</v>
-      </c>
-      <c r="C26" t="n">
-        <v>7</v>
-      </c>
-      <c r="D26" t="n">
-        <v>31.29</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D27" t="n">
-        <v>9.390000000000001</v>
+        <v>244.85</v>
       </c>
       <c r="E27" t="n">
-        <v>9.390000000000001</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="n">
+        <v>36.63</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" t="n">
+        <v>29</v>
+      </c>
+      <c r="D29" t="n">
+        <v>254.7</v>
+      </c>
+      <c r="E29" t="n">
+        <v>254.7</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>4.5</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4.89</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>9</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" t="n">
+        <v>67.66</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" t="n">
+        <v>6</v>
+      </c>
+      <c r="D35" t="n">
+        <v>60.11</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D36" t="n">
-        <v>9.390000000000001</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>55.62</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>9</v>
+      </c>
+      <c r="C37" t="n">
+        <v>9</v>
+      </c>
+      <c r="D37" t="n">
+        <v>71.31</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
-        <v>4.5</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D40" t="n">
-        <v>4.89</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>92.27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>17</v>
+      </c>
+      <c r="C41" t="n">
+        <v>17</v>
+      </c>
+      <c r="D41" t="n">
+        <v>162.43</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2</v>
-      </c>
-      <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="n">
-        <v>9.390000000000001</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>4.89</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
-        <v>4.5</v>
+        <v>54.43</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D47" t="n">
-        <v>4.89</v>
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D48" t="n">
+        <v>63.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>45.58</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>30</v>
+      </c>
+      <c r="C52" t="n">
+        <v>29</v>
+      </c>
+      <c r="D52" t="n">
+        <v>254.7</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>17</v>
+      </c>
+      <c r="C55" t="n">
+        <v>16</v>
+      </c>
+      <c r="D55" t="n">
+        <v>135.16</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8</v>
+      </c>
+      <c r="D56" t="n">
+        <v>73.90000000000001</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" t="n">
+        <v>33.94</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" t="n">
-        <v>9.390000000000001</v>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>23.01</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>26</v>
+      </c>
+      <c r="C62" t="n">
+        <v>25</v>
+      </c>
+      <c r="D62" t="n">
+        <v>231.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-08-31 17:47
</commit_message>
<xml_diff>
--- a/reports/2026-08-31.xlsx
+++ b/reports/2026-08-31.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1762,6 +1762,135 @@
       </c>
       <c r="K31" t="n">
         <v>16.14</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-31T13:43:31.728934+00:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="G32" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-0.0011</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>10.12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-31T14:48:52.954816+00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F33" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="G33" t="n">
+        <v>34.83</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>-18.11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-31T14:56:54.532380+00:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F34" t="n">
+        <v>17.21</v>
+      </c>
+      <c r="G34" t="n">
+        <v>31.28</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.00149</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>14.07</v>
       </c>
     </row>
   </sheetData>
@@ -1775,7 +1904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1797,7 +1926,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -1807,7 +1936,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -1817,7 +1946,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1827,7 +1956,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.9393939393939394</v>
       </c>
     </row>
     <row r="6">
@@ -1837,7 +1966,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>254.7</v>
+        <v>260.78</v>
       </c>
     </row>
     <row r="7">
@@ -1847,7 +1976,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>262.76</v>
+        <v>286.95</v>
       </c>
     </row>
     <row r="8">
@@ -1857,7 +1986,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-8.06</v>
+        <v>-26.17</v>
       </c>
     </row>
     <row r="9">
@@ -1867,7 +1996,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32.6</v>
+        <v>10.96</v>
       </c>
     </row>
     <row r="10">
@@ -1877,7 +2006,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>352.1199999999999</v>
+        <v>358.1999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1928,16 +2057,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C15" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="D15" t="n">
-        <v>186.6</v>
+        <v>302.79</v>
       </c>
       <c r="E15" t="n">
-        <v>92.27</v>
+        <v>116.46</v>
       </c>
     </row>
     <row r="16">
@@ -1947,16 +2076,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" t="n">
         <v>36</v>
       </c>
       <c r="D16" t="n">
-        <v>349.58</v>
+        <v>331.47</v>
       </c>
       <c r="E16" t="n">
-        <v>162.43</v>
+        <v>144.32</v>
       </c>
     </row>
     <row r="17">
@@ -1973,13 +2102,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D18" t="n">
-        <v>142.49</v>
+        <v>189.42</v>
       </c>
       <c r="E18" t="n">
         <v>67.66</v>
@@ -1992,16 +2121,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C19" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D19" t="n">
-        <v>143.76</v>
+        <v>153.75</v>
       </c>
       <c r="E19" t="n">
-        <v>60.11</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="20">
@@ -2011,16 +2140,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>92.04000000000001</v>
+        <v>117.94</v>
       </c>
       <c r="E20" t="n">
-        <v>55.62</v>
+        <v>37.51</v>
       </c>
     </row>
     <row r="21">
@@ -2030,13 +2159,13 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>23</v>
+      </c>
+      <c r="C21" t="n">
         <v>22</v>
       </c>
-      <c r="C21" t="n">
-        <v>21</v>
-      </c>
       <c r="D21" t="n">
-        <v>157.89</v>
+        <v>173.15</v>
       </c>
       <c r="E21" t="n">
         <v>71.31</v>
@@ -2056,16 +2185,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C23" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D23" t="n">
-        <v>529.55</v>
+        <v>602.58</v>
       </c>
       <c r="E23" t="n">
-        <v>254.7</v>
+        <v>250.66</v>
       </c>
     </row>
     <row r="24">
@@ -2075,16 +2204,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>3.43</v>
+        <v>17.26</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="25">
@@ -2094,13 +2223,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>3.2</v>
+        <v>14.42</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -2120,13 +2249,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C27" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D27" t="n">
-        <v>244.85</v>
+        <v>275.72</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -2139,13 +2268,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C28" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D28" t="n">
-        <v>36.63</v>
+        <v>94.05</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -2158,16 +2287,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C29" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D29" t="n">
-        <v>254.7</v>
+        <v>264.49</v>
       </c>
       <c r="E29" t="n">
-        <v>254.7</v>
+        <v>260.78</v>
       </c>
     </row>
     <row r="31">
@@ -2222,13 +2351,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>60.11</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="36">
@@ -2238,13 +2367,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C36" t="n">
         <v>6</v>
       </c>
       <c r="D36" t="n">
-        <v>55.62</v>
+        <v>37.51</v>
       </c>
     </row>
     <row r="37">
@@ -2292,13 +2421,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C40" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>92.27</v>
+        <v>116.46</v>
       </c>
     </row>
     <row r="41">
@@ -2308,13 +2437,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C41" t="n">
         <v>17</v>
       </c>
       <c r="D41" t="n">
-        <v>162.43</v>
+        <v>144.32</v>
       </c>
     </row>
     <row r="43">
@@ -2435,156 +2564,166 @@
         <v>45.58</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>10.12</v>
+      </c>
+    </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-4.04</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>30</v>
-      </c>
-      <c r="C52" t="n">
-        <v>29</v>
-      </c>
-      <c r="D52" t="n">
-        <v>254.7</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>32</v>
+      </c>
+      <c r="C54" t="n">
+        <v>30</v>
+      </c>
+      <c r="D54" t="n">
+        <v>250.66</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C55" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>135.16</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>8</v>
-      </c>
-      <c r="C56" t="n">
-        <v>8</v>
-      </c>
-      <c r="D56" t="n">
-        <v>73.90000000000001</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" t="n">
-        <v>11.7</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0.20%+</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D58" t="n">
-        <v>33.94</v>
+        <v>127.17</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>9</v>
+      </c>
+      <c r="C59" t="n">
+        <v>9</v>
+      </c>
+      <c r="D59" t="n">
+        <v>87.97</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>11.7</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>0.20%+</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2594,23 +2733,61 @@
         <v>4</v>
       </c>
       <c r="D61" t="n">
-        <v>23.01</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
+        <v>33.94</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="n">
+        <v>33.13</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>28</v>
+      </c>
+      <c r="C65" t="n">
         <v>26</v>
       </c>
-      <c r="C62" t="n">
-        <v>25</v>
-      </c>
-      <c r="D62" t="n">
-        <v>231.69</v>
+      <c r="D65" t="n">
+        <v>227.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-08-31 23:46
</commit_message>
<xml_diff>
--- a/reports/2026-08-31.xlsx
+++ b/reports/2026-08-31.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1891,6 +1891,49 @@
       </c>
       <c r="K34" t="n">
         <v>14.07</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-31T23:26:16.269564+00:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>15</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F35" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.00117</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>8.68</v>
       </c>
     </row>
   </sheetData>
@@ -1904,7 +1947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1926,7 +1969,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -1936,7 +1979,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -1956,7 +1999,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.9411764705882353</v>
       </c>
     </row>
     <row r="6">
@@ -1966,7 +2009,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>260.78</v>
+        <v>269.46</v>
       </c>
     </row>
     <row r="7">
@@ -1976,7 +2019,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>286.95</v>
+        <v>295.63</v>
       </c>
     </row>
     <row r="8">
@@ -1996,7 +2039,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10.96</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="10">
@@ -2006,7 +2049,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>358.1999999999999</v>
+        <v>366.8799999999999</v>
       </c>
     </row>
     <row r="12">
@@ -2057,16 +2100,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D15" t="n">
-        <v>302.79</v>
+        <v>351.73</v>
       </c>
       <c r="E15" t="n">
-        <v>116.46</v>
+        <v>125.14</v>
       </c>
     </row>
     <row r="16">
@@ -2076,13 +2119,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C16" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D16" t="n">
-        <v>331.47</v>
+        <v>348.68</v>
       </c>
       <c r="E16" t="n">
         <v>144.32</v>
@@ -2102,16 +2145,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D18" t="n">
-        <v>189.42</v>
+        <v>223.16</v>
       </c>
       <c r="E18" t="n">
-        <v>67.66</v>
+        <v>76.34</v>
       </c>
     </row>
     <row r="19">
@@ -2121,13 +2164,13 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" t="n">
         <v>19</v>
       </c>
-      <c r="C19" t="n">
-        <v>18</v>
-      </c>
       <c r="D19" t="n">
-        <v>153.75</v>
+        <v>170.28</v>
       </c>
       <c r="E19" t="n">
         <v>84.3</v>
@@ -2140,13 +2183,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C20" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D20" t="n">
-        <v>117.94</v>
+        <v>151.73</v>
       </c>
       <c r="E20" t="n">
         <v>37.51</v>
@@ -2159,13 +2202,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C21" t="n">
         <v>22</v>
       </c>
       <c r="D21" t="n">
-        <v>173.15</v>
+        <v>155.24</v>
       </c>
       <c r="E21" t="n">
         <v>71.31</v>
@@ -2185,16 +2228,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C23" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D23" t="n">
-        <v>602.58</v>
+        <v>668.73</v>
       </c>
       <c r="E23" t="n">
-        <v>250.66</v>
+        <v>259.34</v>
       </c>
     </row>
     <row r="24">
@@ -2249,13 +2292,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C27" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D27" t="n">
-        <v>275.72</v>
+        <v>310.16</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -2268,13 +2311,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C28" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>94.05</v>
+        <v>109.23</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -2287,16 +2330,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C29" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D29" t="n">
-        <v>264.49</v>
+        <v>281.02</v>
       </c>
       <c r="E29" t="n">
-        <v>260.78</v>
+        <v>269.46</v>
       </c>
     </row>
     <row r="31">
@@ -2335,13 +2378,13 @@
         </is>
       </c>
       <c r="B34" t="n">
+        <v>10</v>
+      </c>
+      <c r="C34" t="n">
         <v>9</v>
       </c>
-      <c r="C34" t="n">
-        <v>8</v>
-      </c>
       <c r="D34" t="n">
-        <v>67.66</v>
+        <v>76.34</v>
       </c>
     </row>
     <row r="35">
@@ -2421,13 +2464,13 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>16</v>
+      </c>
+      <c r="C40" t="n">
         <v>15</v>
       </c>
-      <c r="C40" t="n">
-        <v>14</v>
-      </c>
       <c r="D40" t="n">
-        <v>116.46</v>
+        <v>125.14</v>
       </c>
     </row>
     <row r="41">
@@ -2596,198 +2639,214 @@
         <v>-4.04</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>8.68</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>32</v>
-      </c>
-      <c r="C54" t="n">
-        <v>30</v>
-      </c>
-      <c r="D54" t="n">
-        <v>250.66</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>33</v>
+      </c>
+      <c r="C55" t="n">
+        <v>31</v>
+      </c>
+      <c r="D55" t="n">
+        <v>259.34</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B56" t="n">
         <v>1</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C56" t="n">
         <v>1</v>
       </c>
-      <c r="D55" t="n">
+      <c r="D56" t="n">
         <v>10.12</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>19</v>
-      </c>
-      <c r="C58" t="n">
-        <v>17</v>
-      </c>
-      <c r="D58" t="n">
-        <v>127.17</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="C59" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D59" t="n">
-        <v>87.97</v>
+        <v>135.85</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>11.7</v>
+        <v>87.97</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>0.20%+</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="B62" t="n">
         <v>4</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C62" t="n">
         <v>4</v>
       </c>
-      <c r="D61" t="n">
+      <c r="D62" t="n">
         <v>33.94</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>5</v>
-      </c>
-      <c r="C64" t="n">
-        <v>5</v>
-      </c>
-      <c r="D64" t="n">
-        <v>33.13</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="C65" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="D65" t="n">
-        <v>227.65</v>
+        <v>33.13</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>29</v>
+      </c>
+      <c r="C66" t="n">
+        <v>27</v>
+      </c>
+      <c r="D66" t="n">
+        <v>236.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>